<commit_message>
m a j du 21-03
</commit_message>
<xml_diff>
--- a/Modele/resultats_XGBoost_Oui (DDBS - euclidean, geometric)_preprocessed_iris_dataset.xlsx
+++ b/Modele/resultats_XGBoost_Oui (DDBS - euclidean, geometric)_preprocessed_iris_dataset.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q9"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -979,6 +979,470 @@
         <v>1</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Oui (DDBS - euclidean, geometric)</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D10" t="n">
+        <v>15</v>
+      </c>
+      <c r="E10" t="n">
+        <v>80</v>
+      </c>
+      <c r="F10" t="n">
+        <v>20</v>
+      </c>
+      <c r="G10" t="n">
+        <v>20</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>{'learning_rate': 0.1, 'max_depth': 6, 'n_estimators': 100}</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>{'n_estimators': 208, 'max_depth': 12, 'learning_rate': 0.015630429834672988}</t>
+        </is>
+      </c>
+      <c r="O10" t="n">
+        <v>1</v>
+      </c>
+      <c r="P10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Oui (DDBS - euclidean, geometric)</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D11" t="n">
+        <v>15</v>
+      </c>
+      <c r="E11" t="n">
+        <v>80</v>
+      </c>
+      <c r="F11" t="n">
+        <v>20</v>
+      </c>
+      <c r="G11" t="n">
+        <v>20</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>{'learning_rate': 0.1, 'max_depth': 6, 'n_estimators': 100}</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.9501253132832079</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>{'n_estimators': 78, 'max_depth': 20, 'learning_rate': 0.013296649493591259}</t>
+        </is>
+      </c>
+      <c r="O11" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0.9501253132832079</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Oui (DDBS - euclidean, geometric)</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="D12" t="n">
+        <v>15</v>
+      </c>
+      <c r="E12" t="n">
+        <v>80</v>
+      </c>
+      <c r="F12" t="n">
+        <v>20</v>
+      </c>
+      <c r="G12" t="n">
+        <v>20</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>{'learning_rate': 0.1, 'max_depth': 6, 'n_estimators': 100}</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.9506666666666668</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>{'n_estimators': 164, 'max_depth': 14, 'learning_rate': 0.13080786575664843}</t>
+        </is>
+      </c>
+      <c r="O12" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0.9506666666666668</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Oui (DDBS - euclidean, geometric)</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D13" t="n">
+        <v>15</v>
+      </c>
+      <c r="E13" t="n">
+        <v>80</v>
+      </c>
+      <c r="F13" t="n">
+        <v>20</v>
+      </c>
+      <c r="G13" t="n">
+        <v>20</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>{'learning_rate': 0.1, 'max_depth': 6, 'n_estimators': 100}</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="K13" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>{'n_estimators': 366, 'max_depth': 14, 'learning_rate': 0.08202622929561816}</t>
+        </is>
+      </c>
+      <c r="O13" t="n">
+        <v>1</v>
+      </c>
+      <c r="P13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Oui (DDBS - euclidean, geometric)</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D14" t="n">
+        <v>16</v>
+      </c>
+      <c r="E14" t="n">
+        <v>80</v>
+      </c>
+      <c r="F14" t="n">
+        <v>20</v>
+      </c>
+      <c r="G14" t="n">
+        <v>20</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>{'learning_rate': 0.1, 'max_depth': 6, 'n_estimators': 100}</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="K14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>{'n_estimators': 163, 'max_depth': 7, 'learning_rate': 0.024739858555679808}</t>
+        </is>
+      </c>
+      <c r="O14" t="n">
+        <v>1</v>
+      </c>
+      <c r="P14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>2</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Oui (DDBS - euclidean, geometric)</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D15" t="n">
+        <v>15</v>
+      </c>
+      <c r="E15" t="n">
+        <v>80</v>
+      </c>
+      <c r="F15" t="n">
+        <v>20</v>
+      </c>
+      <c r="G15" t="n">
+        <v>20</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>{'learning_rate': 0.1, 'max_depth': 6, 'n_estimators': 100}</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0.9503836317135551</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>{'n_estimators': 270, 'max_depth': 20, 'learning_rate': 0.02738760482297254}</t>
+        </is>
+      </c>
+      <c r="O15" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0.9503836317135551</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Oui (DDBS - euclidean, geometric)</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D16" t="n">
+        <v>16</v>
+      </c>
+      <c r="E16" t="n">
+        <v>16</v>
+      </c>
+      <c r="F16" t="n">
+        <v>20</v>
+      </c>
+      <c r="G16" t="n">
+        <v>20</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>{'learning_rate': 0.1, 'max_depth': 6, 'n_estimators': 100}</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.949874686716792</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>{'n_estimators': 395, 'max_depth': 9, 'learning_rate': 0.0918265535647125}</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0.949874686716792</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>2</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Oui (DDBS - euclidean, geometric)</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D17" t="n">
+        <v>15</v>
+      </c>
+      <c r="E17" t="n">
+        <v>15</v>
+      </c>
+      <c r="F17" t="n">
+        <v>20</v>
+      </c>
+      <c r="G17" t="n">
+        <v>20</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>{'learning_rate': 0.1, 'max_depth': 6, 'n_estimators': 100}</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="K17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>{'n_estimators': 494, 'max_depth': 10, 'learning_rate': 0.031203742369498855}</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>1</v>
+      </c>
+      <c r="P17" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>